<commit_message>
Add 49 red base recipes excel/csv data file
</commit_message>
<xml_diff>
--- a/Base_Recipes_Template.xlsx
+++ b/Base_Recipes_Template.xlsx
@@ -1,62 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <bookViews>
-    <workbookView xWindow="130" yWindow="490" windowWidth="18880" windowHeight="8740"/>
-  </bookViews>
   <sheets>
     <sheet name="Base Recipes Template" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
-  <si>
-    <t>recipeName</t>
-  </si>
-  <si>
-    <t>batchYield</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>ingredientName</t>
-  </si>
-  <si>
-    <t>qty</t>
-  </si>
-  <si>
-    <t>Tomato Chutney Base</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>Organic Tomato</t>
-  </si>
-  <si>
-    <t>Wood Pressed Groundnut Oil</t>
-  </si>
-  <si>
-    <t>Dosa Batter Base</t>
-  </si>
-  <si>
-    <t>Foxtail Millet</t>
-  </si>
-  <si>
-    <t>BANG BANG CAULIFLOWER Batter 1 potion</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -93,11 +72,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -422,89 +396,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.08203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.9140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.75" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>recipeName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>batchYield</v>
+      </c>
+      <c r="C1" t="str">
+        <v>unit</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ingredientName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>qty</v>
+      </c>
+      <c r="F1" t="str">
+        <v>gramsMl</v>
+      </c>
+      <c r="G1" t="str">
+        <v>uom</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>11</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>HIGH PROTEIN PASTA SAUCE</v>
       </c>
       <c r="B2">
+        <v>3100</v>
+      </c>
+      <c r="C2" t="str">
+        <v>GRM</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TOMATO</v>
+      </c>
+      <c r="E2">
+        <v>1500</v>
+      </c>
+      <c r="F2">
+        <v>1500</v>
+      </c>
+      <c r="G2" t="str">
+        <v>GRM</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>HIGH PROTEIN PASTA SAUCE</v>
+      </c>
+      <c r="B3">
+        <v>3100</v>
+      </c>
+      <c r="C3" t="str">
+        <v>GRM</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Organic Cinnamon Powder</v>
+      </c>
+      <c r="E3">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="F3">
         <v>5</v>
       </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4">
-        <v>6</v>
+      <c r="G3" t="str">
+        <v>GRM</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A3:E4 B2:E2" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>